<commit_message>
Improve investor matching: check-range filter, email column, robust JSON errors
- investor_utils: add parseRevenueToMillions/parseInvestorCheckRange/extractRevenueFromPayload helpers and use them in rankInvestorsByRelevance for hard filtering by deal scale and startup bonus when revenue is missing
- investor_utils: load email column (D) from rag_investors.xlsx and render it on investor cards (mailto link or placeholder text)
- investor_utils + public_investor_match: extend formatInvestorReason and AI prompts to mention revenue scale / startup preference, with fallback to relaxed ranking when too few candidates pass the filter
- investor-match (frontend): replace HTML5 pattern validation with friendly JS messages and tolerate non-JSON server responses
- public_investor_match: add shutdown/error/try-catch wrappers so any PHP error returns a valid JSON 500 instead of HTML

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/rag_investors.xlsx
+++ b/rag_investors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vitalyvinogradov/INVESTORS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vitalyvinogradov/SmartBizSell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0DAE02A-73C9-5A42-8A42-3CA2478EA102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582A7C90-0371-9246-8CC8-A6A530151A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4380" yWindow="580" windowWidth="24420" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="438">
   <si>
     <t>Название</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Агросектор, производство продуктов питания</t>
   </si>
   <si>
-    <t>Не указано</t>
-  </si>
-  <si>
     <t>Московская биржа</t>
   </si>
   <si>
@@ -272,9 +269,6 @@
     <t>Потребительский сектор, софт, фарма, частная медицина, финтех, онлайн-сервисы</t>
   </si>
   <si>
-    <t>0,5–1,5 млрд руб. (Pre-IPO), от 2,5 млрд руб. (клубные сделки)</t>
-  </si>
-  <si>
     <t>Константин Ладыгин</t>
   </si>
   <si>
@@ -290,9 +284,6 @@
     <t>СБЕР</t>
   </si>
   <si>
-    <t>IT, финтех, онлайн-сервисы, недвижимость, промышленность, агросектор, медицина, фарма</t>
-  </si>
-  <si>
     <t>Восток Инвестиции / ex-Baring Vostok</t>
   </si>
   <si>
@@ -659,9 +650,6 @@
     <t>IT, маркетплейсы, непродовольственный ритейл</t>
   </si>
   <si>
-    <t>От 2–3 млрд руб. EBITDA (для LP)</t>
-  </si>
-  <si>
     <t>Ташир</t>
   </si>
   <si>
@@ -785,9 +773,6 @@
     <t>Производство, химия, фарма, клиники, ритейл, логистика</t>
   </si>
   <si>
-    <t>От 3 млрд руб. выручки, EBITDA ≥30%</t>
-  </si>
-  <si>
     <t>Волга Групп</t>
   </si>
   <si>
@@ -828,13 +813,535 @@
   </si>
   <si>
     <t>Крупные сделки</t>
+  </si>
+  <si>
+    <t>ФРИИ</t>
+  </si>
+  <si>
+    <t>IT-стартапы, цифровые сервисы, интернет-проекты</t>
+  </si>
+  <si>
+    <t>От 3–15 млн ₽ (pre-seed / seed)</t>
+  </si>
+  <si>
+    <t>Технологические компании Москвы</t>
+  </si>
+  <si>
+    <t>От 20–150 млн ₽ (seed и рост)</t>
+  </si>
+  <si>
+    <t>Impact Capital</t>
+  </si>
+  <si>
+    <t>Малый и средний бизнес (без жёсткой отраслевой фокусировки)</t>
+  </si>
+  <si>
+    <t>$50k – $1M</t>
+  </si>
+  <si>
+    <t>НТИ</t>
+  </si>
+  <si>
+    <t>Deeptech, ИИ, БПЛА, микроэлектроника, новые материалы, цифровая медицина</t>
+  </si>
+  <si>
+    <t>От 30 млн до нескольких сотен млн ₽</t>
+  </si>
+  <si>
+    <t>Iskra Ventures</t>
+  </si>
+  <si>
+    <t>Consumer, e-commerce, video &amp; content, mobility</t>
+  </si>
+  <si>
+    <t>Seed / Early Stage</t>
+  </si>
+  <si>
+    <t>Телеком, IT, проекты экосистемы Билайн</t>
+  </si>
+  <si>
+    <t>Не публикуется (корпоративный венчур)</t>
+  </si>
+  <si>
+    <t>Malina VC</t>
+  </si>
+  <si>
+    <t>Fintech, marketplaces</t>
+  </si>
+  <si>
+    <t>Seed / Growth (фонд ~1 млрд ₽)</t>
+  </si>
+  <si>
+    <t>Friends VC</t>
+  </si>
+  <si>
+    <t>B2B Software, зрелые технологические компании</t>
+  </si>
+  <si>
+    <t>От 50–300+ млн ₽ (late seed / A–B)</t>
+  </si>
+  <si>
+    <t>Восход</t>
+  </si>
+  <si>
+    <t>Deeptech, микроэлектроника, ИИ, робототехника, промышленные технологии</t>
+  </si>
+  <si>
+    <t>Потребительские рынки, платформы, retail, игры, мода</t>
+  </si>
+  <si>
+    <t>До нескольких десятков млн ₽</t>
+  </si>
+  <si>
+    <t>СТ Капитал</t>
+  </si>
+  <si>
+    <t>Быстрорастущие технологические компании</t>
+  </si>
+  <si>
+    <t>Softline Venture</t>
+  </si>
+  <si>
+    <t>IT, software, технологические компании</t>
+  </si>
+  <si>
+    <t>Сигнал</t>
+  </si>
+  <si>
+    <t>Масштабирование технологических проектов</t>
+  </si>
+  <si>
+    <t>Skolkovo VC</t>
+  </si>
+  <si>
+    <t>High-tech стартапы (экосистема Сколково)</t>
+  </si>
+  <si>
+    <t>Early / Growth stage</t>
+  </si>
+  <si>
+    <t>Lanit Ventures</t>
+  </si>
+  <si>
+    <t>IT и интернет-проекты</t>
+  </si>
+  <si>
+    <t>Early stage</t>
+  </si>
+  <si>
+    <t>Stamina VC</t>
+  </si>
+  <si>
+    <t>Технологические компании (early / growth)</t>
+  </si>
+  <si>
+    <t>Десятки — сотни млн ₽</t>
+  </si>
+  <si>
+    <t>3 Streams</t>
+  </si>
+  <si>
+    <t>Потребительские бренды, lifestyle, быстрорастущие компании</t>
+  </si>
+  <si>
+    <t>От 150+ млн ₽ выручки (private equity)</t>
+  </si>
+  <si>
+    <t>email для отправки тизер</t>
+  </si>
+  <si>
+    <t>invest@goodnessfoods.ru</t>
+  </si>
+  <si>
+    <t>(нет публичного)</t>
+  </si>
+  <si>
+    <t>От 300 млн руб. (growth / PE)</t>
+  </si>
+  <si>
+    <t>invest@moex.com</t>
+  </si>
+  <si>
+    <t>50–300 млн руб.</t>
+  </si>
+  <si>
+    <t>invest@alteracapital.ru</t>
+  </si>
+  <si>
+    <t>invest@kontur.ru</t>
+  </si>
+  <si>
+    <t>flow@kamaflow.com</t>
+  </si>
+  <si>
+    <t>invest@altuscapital.ru</t>
+  </si>
+  <si>
+    <t>invest@pangeocapital.com</t>
+  </si>
+  <si>
+    <t>invest@atollcapital.ru</t>
+  </si>
+  <si>
+    <t>invest@insightgroup.ru</t>
+  </si>
+  <si>
+    <t>100–800 млн руб.</t>
+  </si>
+  <si>
+    <t>invest@k2invest.ru</t>
+  </si>
+  <si>
+    <t>invest@signal.vc</t>
+  </si>
+  <si>
+    <t>invest@briocapital.ru</t>
+  </si>
+  <si>
+    <t>invest@arcticinvest.ru</t>
+  </si>
+  <si>
+    <t>От 500 млн руб. (PE)</t>
+  </si>
+  <si>
+    <t>invest@sinara-group.com</t>
+  </si>
+  <si>
+    <t>invest@sovcombank.ru</t>
+  </si>
+  <si>
+    <t>От 300 млн руб.</t>
+  </si>
+  <si>
+    <t>invest@chernogolovka.ru</t>
+  </si>
+  <si>
+    <t>invest@supplementgroup.ru</t>
+  </si>
+  <si>
+    <t>invest@exponenta.ru</t>
+  </si>
+  <si>
+    <t>От 100–500 млн руб.</t>
+  </si>
+  <si>
+    <t>invest@balchugcapital.ru</t>
+  </si>
+  <si>
+    <t>invest@s8capital.ru</t>
+  </si>
+  <si>
+    <t>invest@sfi.ru</t>
+  </si>
+  <si>
+    <t>invest@privateassets.ru</t>
+  </si>
+  <si>
+    <t>Крупные сделки (от 1 млрд руб.)</t>
+  </si>
+  <si>
+    <t>invest@lukoil.com</t>
+  </si>
+  <si>
+    <t>invest@rossium.ru</t>
+  </si>
+  <si>
+    <t>От 500 млн руб.</t>
+  </si>
+  <si>
+    <t>invest@evolution.ru</t>
+  </si>
+  <si>
+    <t>invest@invellect.ru</t>
+  </si>
+  <si>
+    <t>invest@inweasta.com</t>
+  </si>
+  <si>
+    <t>invest@gs-invest.ru</t>
+  </si>
+  <si>
+    <t>invest@mts.ru</t>
+  </si>
+  <si>
+    <t>invest@agrocomgroup.ru</t>
+  </si>
+  <si>
+    <t>0,5–1,5 млрд руб. (Pre-IPO), от 2,5 млрд (клубные)</t>
+  </si>
+  <si>
+    <t>invest@vim-invest.ru</t>
+  </si>
+  <si>
+    <t>От 200 млн руб.</t>
+  </si>
+  <si>
+    <t>IT, финтех, онлайн-сервисы, недвижимость, промышленность, агросектор, медицина</t>
+  </si>
+  <si>
+    <t>Крупные сделки (от 500 млн руб.)</t>
+  </si>
+  <si>
+    <t>invest@sber.ru</t>
+  </si>
+  <si>
+    <t>invest@east-west.vc</t>
+  </si>
+  <si>
+    <t>invest@rdif.ru</t>
+  </si>
+  <si>
+    <t>invest@pfpg.ru</t>
+  </si>
+  <si>
+    <t>invest@medinvestgroup.ru</t>
+  </si>
+  <si>
+    <t>invest@talosfund.ru</t>
+  </si>
+  <si>
+    <t>invest@afk.system.ru</t>
+  </si>
+  <si>
+    <t>invest@bonumcapital.ru</t>
+  </si>
+  <si>
+    <t>invest@severgroup.ru</t>
+  </si>
+  <si>
+    <t>invest@aeon.ru</t>
+  </si>
+  <si>
+    <t>invest@eskadra.ru</t>
+  </si>
+  <si>
+    <t>iz@tealtechcapital.com</t>
+  </si>
+  <si>
+    <t>invest@agranta.ru</t>
+  </si>
+  <si>
+    <t>invest@akropol.ru</t>
+  </si>
+  <si>
+    <t>invest@renova.ru</t>
+  </si>
+  <si>
+    <t>invest@ream.ru</t>
+  </si>
+  <si>
+    <t>invest@interrao.ru</t>
+  </si>
+  <si>
+    <t>invest@basic-element.ru</t>
+  </si>
+  <si>
+    <t>invest@indigocapital.ru</t>
+  </si>
+  <si>
+    <t>invest@sds-group.ru</t>
+  </si>
+  <si>
+    <t>invest@ugmk.com</t>
+  </si>
+  <si>
+    <t>invest@fosun.com</t>
+  </si>
+  <si>
+    <t>invest@isrholding.ru</t>
+  </si>
+  <si>
+    <t>invest@sindika.ru</t>
+  </si>
+  <si>
+    <t>invest@rota.ru</t>
+  </si>
+  <si>
+    <t>invest@ekto.ru</t>
+  </si>
+  <si>
+    <t>invest@mubadala.ae</t>
+  </si>
+  <si>
+    <t>invest@agrokplex.ru</t>
+  </si>
+  <si>
+    <t>invest@marathongroup.ru</t>
+  </si>
+  <si>
+    <t>invest@strongbow.ru</t>
+  </si>
+  <si>
+    <t>invest@russianfunds.ru</t>
+  </si>
+  <si>
+    <t>invest@kismet.ru</t>
+  </si>
+  <si>
+    <t>invest@gazprombank.ru</t>
+  </si>
+  <si>
+    <t>invest@psm.ru</t>
+  </si>
+  <si>
+    <t>invest@delo-group.ru</t>
+  </si>
+  <si>
+    <t>invest@investag.ru</t>
+  </si>
+  <si>
+    <t>invest@udscapital.ru</t>
+  </si>
+  <si>
+    <t>invest@proximacapital.ru</t>
+  </si>
+  <si>
+    <t>invest@novard.ru</t>
+  </si>
+  <si>
+    <t>invest@geminvest.ru</t>
+  </si>
+  <si>
+    <t>От 2–3 млрд руб. EBITDA</t>
+  </si>
+  <si>
+    <t>invest@m9capital.ru</t>
+  </si>
+  <si>
+    <t>invest@tashir.ru</t>
+  </si>
+  <si>
+    <t>invest@n3.group</t>
+  </si>
+  <si>
+    <t>invest@x2.ru</t>
+  </si>
+  <si>
+    <t>invest@adamant.ru</t>
+  </si>
+  <si>
+    <t>invest@huaren.ru</t>
+  </si>
+  <si>
+    <t>invest@a-nn.ru</t>
+  </si>
+  <si>
+    <t>invest@generalinvest.ru</t>
+  </si>
+  <si>
+    <t>invest@osnovacapital.ru</t>
+  </si>
+  <si>
+    <t>invest@stroma.ru</t>
+  </si>
+  <si>
+    <t>invest@voskhod.vc</t>
+  </si>
+  <si>
+    <t>invest@skcapital.ru</t>
+  </si>
+  <si>
+    <t>invest@trinfico.ru</t>
+  </si>
+  <si>
+    <t>invest@1147group.ru</t>
+  </si>
+  <si>
+    <t>invest@alfin.am</t>
+  </si>
+  <si>
+    <t>invest@cfcm.ru</t>
+  </si>
+  <si>
+    <t>invest@fordewind.ru</t>
+  </si>
+  <si>
+    <t>От 3 млрд руб. выручки</t>
+  </si>
+  <si>
+    <t>invest@aquilainvest.ru</t>
+  </si>
+  <si>
+    <t>invest@volga-group.ru</t>
+  </si>
+  <si>
+    <t>invest@alfagroup.ru</t>
+  </si>
+  <si>
+    <t>invest@phystechventures.ru</t>
+  </si>
+  <si>
+    <t>invest@ucm.ru</t>
+  </si>
+  <si>
+    <t>invest@polyus.com</t>
+  </si>
+  <si>
+    <t>partners@frii.ru</t>
+  </si>
+  <si>
+    <t>МВФ (Московский венчурный фонд)</t>
+  </si>
+  <si>
+    <t>invest@mvf.ru</t>
+  </si>
+  <si>
+    <t>invest@impactcapital.ru</t>
+  </si>
+  <si>
+    <t>info@nti.ru</t>
+  </si>
+  <si>
+    <t>invest@iskraventures.ru</t>
+  </si>
+  <si>
+    <t>Хайв (Hive)</t>
+  </si>
+  <si>
+    <t>startups@bee-hive.ru</t>
+  </si>
+  <si>
+    <t>startups@malina.vc</t>
+  </si>
+  <si>
+    <t>hello@friends.vc</t>
+  </si>
+  <si>
+    <t>100–500+ млн руб.</t>
+  </si>
+  <si>
+    <t>Growth-stage (от 100 млн руб.)</t>
+  </si>
+  <si>
+    <t>invest@stcapital.ru</t>
+  </si>
+  <si>
+    <t>До $1M</t>
+  </si>
+  <si>
+    <t>info@softlinevp.com</t>
+  </si>
+  <si>
+    <t>Growth investments (от 100 млн руб.)</t>
+  </si>
+  <si>
+    <t>invest@skolkovo.vc</t>
+  </si>
+  <si>
+    <t>invest@lanitventures.ru</t>
+  </si>
+  <si>
+    <t>invest@staminavc.ru</t>
+  </si>
+  <si>
+    <t>invest@3streams.ru</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -842,19 +1349,34 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -866,14 +1388,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1211,1339 +1738,2063 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:D140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
     <col min="2" max="2" width="75.33203125" customWidth="1"/>
-    <col min="3" max="3" width="57.6640625" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="D1" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="D2" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="B6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" s="4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" s="4" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="B12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="B13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" s="4" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="B15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" s="4" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="B18" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B19" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C19" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="B20" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="B21" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C22" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="B23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C23" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="B24" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C24" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="B25" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" s="4" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="B26" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C26" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="B27" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="B28" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C28" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="B29" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C29" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="B30" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C30" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C31" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="B32" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" s="4" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="B33" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C33" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="B34" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="B35" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C35" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="B36" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C36" t="s">
+      <c r="B37" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+      <c r="C37" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C37" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="C38" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C38" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="B40" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C40" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C39" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="D40" s="4" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C41" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="B42" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C42" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C41" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="B43" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C43" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C42" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="B44" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C44" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C43" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="B45" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C45" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C44" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="B46" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C46" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="B47" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C47" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C46" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="B48" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C48" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C47" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="D48" s="4" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C49" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="B50" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C50" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C49" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="B51" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C51" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C50" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="B52" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C52" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C51" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="B53" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C53" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C52" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="B54" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C54" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C53" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+      <c r="B55" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C55" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C54" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+      <c r="B56" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C56" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C55" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+      <c r="B57" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C57" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="C56" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+      <c r="B58" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C58" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C57" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="B59" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C59" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C58" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+      <c r="B60" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C60" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C59" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+      <c r="B61" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C61" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C60" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+      <c r="B62" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C62" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C61" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+      <c r="B63" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C63" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C62" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+      <c r="B64" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C64" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C63" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
+      <c r="B65" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C65" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C64" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+      <c r="B66" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C66" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C65" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
+      <c r="B67" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C67" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="C66" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
+      <c r="B68" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C68" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C67" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
+      <c r="B69" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C69" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C68" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+      <c r="B70" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C70" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C69" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+      <c r="B71" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C71" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="C70" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+      <c r="B72" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C72" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C71" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+      <c r="B73" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C73" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C72" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+      <c r="B74" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C74" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C73" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
+      <c r="B75" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C75" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C74" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
+      <c r="B76" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C76" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C75" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
+      <c r="B77" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C77" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C76" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
+      <c r="B78" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C78" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C77" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
+      <c r="B79" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C79" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="C78" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
+      <c r="B80" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C80" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C79" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
+      <c r="B81" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C81" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C80" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
+      <c r="B82" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C82" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C81" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
+      <c r="B83" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C83" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C82" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
+      <c r="B84" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C84" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C83" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
+      <c r="B85" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C85" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="C84" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
+      <c r="D85" s="4" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B86" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C86" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="2" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+      <c r="B87" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C87" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C86" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
+      <c r="B88" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C88" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="C87" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+      <c r="B89" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B88" t="s">
+      <c r="C89" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C88" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+      <c r="B90" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C90" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="C89" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+      <c r="B91" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C91" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C90" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+      <c r="B92" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B91" t="s">
+      <c r="C92" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C91" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+      <c r="B93" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C93" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="C92" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+      <c r="B94" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C94" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C93" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+      <c r="B95" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="B94" t="s">
+      <c r="C95" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C94" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
+      <c r="D95" s="4" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B96" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C96" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" s="2" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
+      <c r="B97" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="B96" t="s">
+      <c r="C97" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="C96" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
+      <c r="B98" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="B97" t="s">
+      <c r="C98" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C97" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
+      <c r="B99" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B98" t="s">
+      <c r="C99" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="C98" t="s">
+      <c r="B100" s="3" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
+      <c r="C100" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B101" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="C99" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+      <c r="C101" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B102" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="C100" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
+      <c r="C102" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B103" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="C101" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
+      <c r="C103" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B104" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="C102" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
+      <c r="C104" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A105" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B105" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C103" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
+      <c r="C105" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A106" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B106" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="C104" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
+      <c r="C106" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A107" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B107" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="C105" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
+      <c r="C107" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="B106" t="s">
+      <c r="D107" s="4" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A108" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C106" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
+      <c r="B108" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="B107" t="s">
+      <c r="C108" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="C107" t="s">
+      <c r="D108" s="4" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A109" s="2" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
+      <c r="B109" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="B108" t="s">
+      <c r="C109" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="C108" t="s">
+      <c r="D109" s="4" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A110" s="2" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
+      <c r="B110" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="B109" t="s">
+      <c r="C110" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="C109" t="s">
+      <c r="D110" s="4" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A111" s="2" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
+      <c r="B111" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="B110" t="s">
+      <c r="C111" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="C110" t="s">
+      <c r="D111" s="4" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A112" s="2" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
+      <c r="B112" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="B111" t="s">
+      <c r="C112" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="C111" t="s">
+      <c r="D112" s="4" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A113" s="2" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
+      <c r="B113" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="B112" t="s">
+      <c r="C113" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="C112" t="s">
+      <c r="D113" s="4" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A114" s="2" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
+      <c r="B114" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="B113" t="s">
+      <c r="C114" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D114" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A115" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C113" t="s">
+      <c r="B115" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
+      <c r="C115" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D115" s="4" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A116" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B116" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="C114" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
+      <c r="C116" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="B115" t="s">
+      <c r="D116" s="4" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A117" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C115" t="s">
+      <c r="B117" s="3" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
+      <c r="C117" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="B116" t="s">
+      <c r="D117" s="4" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A118" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C116" t="s">
+      <c r="B118" s="3" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
+      <c r="C118" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A119" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B119" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="C117" t="s">
+      <c r="C119" s="3" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
+      <c r="D119" s="4" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A120" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B120" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="C118" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
+      <c r="C120" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="B119" t="s">
+      <c r="D120" s="4" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A121" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C119" t="s">
+      <c r="B121" s="3" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
+      <c r="C121" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="B120" t="s">
+      <c r="D121" s="4" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A122" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B122" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="C120" t="s">
+      <c r="C122" s="3" t="s">
         <v>268</v>
       </c>
+      <c r="D122" s="4" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A123" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A124" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="D124" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A125" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="D125" s="4" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A126" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A127" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A128" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D128" s="4" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A129" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D129" s="4" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A130" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="D130" s="4" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A131" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="D131" s="4" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A132" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="D132" s="4" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A133" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="D133" s="4" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A134" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A135" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A136" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A137" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A138" s="1"/>
+      <c r="B138" s="1"/>
+      <c r="C138" s="1"/>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A139" s="1"/>
+      <c r="B139" s="1"/>
+      <c r="C139" s="1"/>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A140" s="1"/>
+      <c r="B140" s="1"/>
+      <c r="C140" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="mailto:invest@goodnessfoods.ru" xr:uid="{0308B25A-8F75-384C-B521-4992BD6C3E1A}"/>
+    <hyperlink ref="D4" r:id="rId2" display="mailto:invest@moex.com" xr:uid="{5C7FA27E-6422-2443-846F-E68A2CFDC134}"/>
+    <hyperlink ref="D5" r:id="rId3" display="mailto:invest@alteracapital.ru" xr:uid="{6EC236B2-3951-7442-9C76-CC61A9FAB1F7}"/>
+    <hyperlink ref="D6" r:id="rId4" display="mailto:invest@kontur.ru" xr:uid="{D60F660B-0ED6-B141-B141-6E2308AD0BD5}"/>
+    <hyperlink ref="D7" r:id="rId5" display="mailto:flow@kamaflow.com" xr:uid="{08F24D1D-CC6F-124A-B2EE-C5C1ACA5E3C0}"/>
+    <hyperlink ref="D8" r:id="rId6" display="mailto:invest@altuscapital.ru" xr:uid="{D1C15CF8-6E0B-8C45-B37B-4BF9A73DFA6E}"/>
+    <hyperlink ref="D11" r:id="rId7" display="mailto:invest@pangeocapital.com" xr:uid="{AA198327-F56B-AF41-893D-645B731526EE}"/>
+    <hyperlink ref="D12" r:id="rId8" display="mailto:invest@atollcapital.ru" xr:uid="{A40E5656-EB40-F745-BDA8-CCBFCF266079}"/>
+    <hyperlink ref="D13" r:id="rId9" display="mailto:invest@insightgroup.ru" xr:uid="{184B6158-D830-8747-9B80-6C63E21B1E89}"/>
+    <hyperlink ref="D14" r:id="rId10" display="mailto:invest@k2invest.ru" xr:uid="{815E1675-03FE-4447-84C6-934672F5A79F}"/>
+    <hyperlink ref="D15" r:id="rId11" display="mailto:invest@signal.vc" xr:uid="{85B1DDFB-A7FC-C14F-ADFC-C811C2164F9B}"/>
+    <hyperlink ref="D16" r:id="rId12" display="mailto:invest@briocapital.ru" xr:uid="{FF8C8335-A557-0849-809F-09392C3757DA}"/>
+    <hyperlink ref="D17" r:id="rId13" display="mailto:invest@arcticinvest.ru" xr:uid="{DB263810-7894-C240-B8CB-40D937CB30C9}"/>
+    <hyperlink ref="D18" r:id="rId14" display="mailto:invest@sinara-group.com" xr:uid="{5844DCED-8F74-0C42-8C6C-E5F4954AAEBD}"/>
+    <hyperlink ref="D19" r:id="rId15" display="mailto:invest@sovcombank.ru" xr:uid="{5E53F7C5-457D-3944-83CC-7FF1948CB53C}"/>
+    <hyperlink ref="D20" r:id="rId16" display="mailto:invest@chernogolovka.ru" xr:uid="{E7838103-E5C7-FD40-B3E2-63FAAEFCFA34}"/>
+    <hyperlink ref="D21" r:id="rId17" display="mailto:invest@supplementgroup.ru" xr:uid="{2F8EF9B2-2C09-2E45-A581-207C10AD0EA0}"/>
+    <hyperlink ref="D22" r:id="rId18" display="mailto:invest@exponenta.ru" xr:uid="{3A8D9A70-82C6-7E43-BD88-F2EA48FF49F0}"/>
+    <hyperlink ref="D24" r:id="rId19" display="mailto:invest@balchugcapital.ru" xr:uid="{12F5BCB4-04F6-F342-9514-FD80BB832DFA}"/>
+    <hyperlink ref="D25" r:id="rId20" display="mailto:invest@s8capital.ru" xr:uid="{86DC554B-027B-E54D-8C5A-F18299EE77CD}"/>
+    <hyperlink ref="D26" r:id="rId21" display="mailto:invest@sfi.ru" xr:uid="{F672158E-E09B-8C4E-AC64-B0557F0C5284}"/>
+    <hyperlink ref="D27" r:id="rId22" display="mailto:invest@privateassets.ru" xr:uid="{491F1D0A-7C25-7C42-9471-9DF4D316E76E}"/>
+    <hyperlink ref="D28" r:id="rId23" display="mailto:invest@lukoil.com" xr:uid="{D0321DA4-30E5-8D4E-B61E-0545F90ED736}"/>
+    <hyperlink ref="D29" r:id="rId24" display="mailto:invest@rossium.ru" xr:uid="{607257D3-A688-B947-BE1F-13BD2064E248}"/>
+    <hyperlink ref="D30" r:id="rId25" display="mailto:invest@evolution.ru" xr:uid="{849E765A-E01C-4149-B9E9-B5B0409ECDF9}"/>
+    <hyperlink ref="D31" r:id="rId26" display="mailto:invest@invellect.ru" xr:uid="{25E6156D-09A7-A849-9B6C-5E3E889EAE72}"/>
+    <hyperlink ref="D32" r:id="rId27" display="mailto:invest@inweasta.com" xr:uid="{423FB96C-62D7-064A-A691-BD955C0D6178}"/>
+    <hyperlink ref="D33" r:id="rId28" display="mailto:invest@gs-invest.ru" xr:uid="{EA054682-01FF-474D-AE8B-FED772C78DE0}"/>
+    <hyperlink ref="D34" r:id="rId29" display="mailto:invest@mts.ru" xr:uid="{2FF0A70E-BA34-654A-98DB-25382BCF3AAA}"/>
+    <hyperlink ref="D35" r:id="rId30" display="mailto:invest@agrocomgroup.ru" xr:uid="{F0E36C6C-A0D9-754E-AE15-BF89C0F38A06}"/>
+    <hyperlink ref="D36" r:id="rId31" display="mailto:invest@vim-invest.ru" xr:uid="{02B79D88-60E0-6746-ABEB-C6FC25F2808E}"/>
+    <hyperlink ref="D39" r:id="rId32" display="mailto:invest@sber.ru" xr:uid="{C8948648-C0CC-D249-A0F6-D50FD35944B0}"/>
+    <hyperlink ref="D40" r:id="rId33" display="mailto:invest@east-west.vc" xr:uid="{103A833A-374A-0348-94F8-EB2638F7CED5}"/>
+    <hyperlink ref="D41" r:id="rId34" display="mailto:invest@rdif.ru" xr:uid="{C67C8AB5-685E-7441-B2B2-16921254857F}"/>
+    <hyperlink ref="D42" r:id="rId35" display="mailto:invest@pfpg.ru" xr:uid="{0F702F1B-5F96-0942-A4F5-25006A1951DE}"/>
+    <hyperlink ref="D43" r:id="rId36" display="mailto:invest@medinvestgroup.ru" xr:uid="{2E55E8AC-CF8F-AD41-82D5-715ED4091E2E}"/>
+    <hyperlink ref="D45" r:id="rId37" display="mailto:invest@talosfund.ru" xr:uid="{97B8F6F0-796C-3146-9C54-88BF5247CAB0}"/>
+    <hyperlink ref="D47" r:id="rId38" display="mailto:invest@afk.system.ru" xr:uid="{8E006A6A-5963-554E-8EA5-1A8D4C650394}"/>
+    <hyperlink ref="D48" r:id="rId39" display="mailto:invest@bonumcapital.ru" xr:uid="{7F3767B0-865D-ED48-A8ED-ABFDBB506D08}"/>
+    <hyperlink ref="D49" r:id="rId40" display="mailto:invest@severgroup.ru" xr:uid="{4A415067-8836-F245-9ACB-CF6D6E4DB1B6}"/>
+    <hyperlink ref="D50" r:id="rId41" display="mailto:invest@aeon.ru" xr:uid="{CFDCF5F8-0758-5F4B-B26B-77E97992F0C0}"/>
+    <hyperlink ref="D53" r:id="rId42" display="mailto:invest@eskadra.ru" xr:uid="{06886096-329B-AA44-B743-FECEF3C33D0B}"/>
+    <hyperlink ref="D56" r:id="rId43" display="mailto:iz@tealtechcapital.com" xr:uid="{51D30589-56F7-964E-8452-156E8ACE682F}"/>
+    <hyperlink ref="D58" r:id="rId44" display="mailto:invest@agranta.ru" xr:uid="{7A26176E-7BBA-D84D-B206-C344F1C3E008}"/>
+    <hyperlink ref="D61" r:id="rId45" display="mailto:invest@akropol.ru" xr:uid="{E5B2AD20-CDE5-E346-9FFD-FE34E252F64F}"/>
+    <hyperlink ref="D62" r:id="rId46" display="mailto:invest@renova.ru" xr:uid="{D0E00A26-93B9-9A44-9F8B-C217609413EA}"/>
+    <hyperlink ref="D64" r:id="rId47" display="mailto:invest@ream.ru" xr:uid="{B3552EF2-2AC5-9E48-9A02-D0D2D3A461D1}"/>
+    <hyperlink ref="D65" r:id="rId48" display="mailto:invest@interrao.ru" xr:uid="{7FE51B79-8D51-E246-85FC-E9B65BAF8114}"/>
+    <hyperlink ref="D66" r:id="rId49" display="mailto:invest@basic-element.ru" xr:uid="{85ED86AA-76E7-3B46-BC8B-F928760ED528}"/>
+    <hyperlink ref="D69" r:id="rId50" display="mailto:invest@indigocapital.ru" xr:uid="{ED21AD22-3A60-C546-B9C4-03D479BE73B4}"/>
+    <hyperlink ref="D70" r:id="rId51" display="mailto:invest@sds-group.ru" xr:uid="{B48553E1-7C15-7547-8FB0-C4D4BD03435E}"/>
+    <hyperlink ref="D71" r:id="rId52" display="mailto:invest@ugmk.com" xr:uid="{390BCE1E-9F45-1B4D-8E08-1D7F9CE2E336}"/>
+    <hyperlink ref="D74" r:id="rId53" display="mailto:invest@fosun.com" xr:uid="{C257C6DD-5369-EF4B-8EDC-0ECCD5516EAF}"/>
+    <hyperlink ref="D75" r:id="rId54" display="mailto:invest@isrholding.ru" xr:uid="{B2354747-663F-4A42-8E09-1F47917F6137}"/>
+    <hyperlink ref="D76" r:id="rId55" display="mailto:invest@sindika.ru" xr:uid="{CE9E689D-D25D-E64C-9C42-68BF2FFF1AD0}"/>
+    <hyperlink ref="D77" r:id="rId56" display="mailto:invest@rota.ru" xr:uid="{1E15E2BB-6348-CF46-9D41-7A74782C8CEB}"/>
+    <hyperlink ref="D78" r:id="rId57" display="mailto:invest@ekto.ru" xr:uid="{B87C453E-B726-A445-9D4E-7F714E36BE82}"/>
+    <hyperlink ref="D79" r:id="rId58" display="mailto:invest@mubadala.ae" xr:uid="{9E8AFFA8-EC42-2D44-85B7-807F427324AE}"/>
+    <hyperlink ref="D80" r:id="rId59" display="mailto:invest@agrokplex.ru" xr:uid="{BB99F2E2-314F-574C-A5AE-DE2D1BF1BA44}"/>
+    <hyperlink ref="D81" r:id="rId60" display="mailto:invest@marathongroup.ru" xr:uid="{67C4E155-BE63-7D47-B892-DAC8E11A9BAD}"/>
+    <hyperlink ref="D83" r:id="rId61" display="mailto:invest@strongbow.ru" xr:uid="{F67EE2EA-A1AF-0049-8424-2FC42391BF46}"/>
+    <hyperlink ref="D84" r:id="rId62" display="mailto:invest@russianfunds.ru" xr:uid="{01D6F963-2765-3449-A059-6D5B21796BC0}"/>
+    <hyperlink ref="D85" r:id="rId63" display="mailto:invest@kismet.ru" xr:uid="{47CC72C3-B2D0-424F-BB46-7B08DD0D2FFA}"/>
+    <hyperlink ref="D88" r:id="rId64" display="mailto:invest@gazprombank.ru" xr:uid="{005AC5E2-47CF-544F-B05B-22A1F5249594}"/>
+    <hyperlink ref="D89" r:id="rId65" display="mailto:invest@psm.ru" xr:uid="{F1414CCD-7647-A949-9B40-FA029E2C9546}"/>
+    <hyperlink ref="D92" r:id="rId66" display="mailto:invest@delo-group.ru" xr:uid="{31CB7907-F9AB-C64E-89E3-5A273EC4EF56}"/>
+    <hyperlink ref="D93" r:id="rId67" display="mailto:invest@investag.ru" xr:uid="{CF3B105F-DDE1-6F41-BB97-DDB98315679F}"/>
+    <hyperlink ref="D94" r:id="rId68" display="mailto:invest@udscapital.ru" xr:uid="{3445329E-F476-3C4A-9EDB-B67B363A79C3}"/>
+    <hyperlink ref="D95" r:id="rId69" display="mailto:invest@proximacapital.ru" xr:uid="{2B37588A-F4DE-5E41-8F51-D35464426536}"/>
+    <hyperlink ref="D96" r:id="rId70" display="mailto:invest@novard.ru" xr:uid="{BB6C12C3-432A-9940-9F99-3FA985F8A84D}"/>
+    <hyperlink ref="D97" r:id="rId71" display="mailto:invest@geminvest.ru" xr:uid="{864D0702-F7E5-764C-A271-1E8CEA7DF380}"/>
+    <hyperlink ref="D98" r:id="rId72" display="mailto:invest@m9capital.ru" xr:uid="{FD39CD29-76A3-B449-8E64-D3E25862B908}"/>
+    <hyperlink ref="D99" r:id="rId73" display="mailto:invest@tashir.ru" xr:uid="{298A28DC-A7FF-794F-957D-7896C5A81D06}"/>
+    <hyperlink ref="D100" r:id="rId74" display="mailto:invest@n3.group" xr:uid="{635BD8C7-EB2B-504D-8476-15CA54D79CC1}"/>
+    <hyperlink ref="D101" r:id="rId75" display="mailto:invest@x2.ru" xr:uid="{B7CD828E-D7D4-EC46-8FBF-C1D16E4B7478}"/>
+    <hyperlink ref="D102" r:id="rId76" display="mailto:invest@adamant.ru" xr:uid="{473D98B2-F246-A14F-B257-3C315C255053}"/>
+    <hyperlink ref="D103" r:id="rId77" display="mailto:invest@huaren.ru" xr:uid="{09FFAAC1-FBE9-A947-AFA9-83184E8ABD2E}"/>
+    <hyperlink ref="D104" r:id="rId78" display="mailto:invest@a-nn.ru" xr:uid="{DE9581CC-55C6-2544-9DD7-542840D80DF5}"/>
+    <hyperlink ref="D105" r:id="rId79" display="mailto:invest@generalinvest.ru" xr:uid="{249B5669-9357-0547-9925-DCB63275A0E9}"/>
+    <hyperlink ref="D106" r:id="rId80" display="mailto:invest@osnovacapital.ru" xr:uid="{4634CE15-5F71-BC4D-842E-47B83A46EA3E}"/>
+    <hyperlink ref="D107" r:id="rId81" display="mailto:invest@stroma.ru" xr:uid="{47452EEF-BD9E-FD42-8027-A4B5029B1A33}"/>
+    <hyperlink ref="D108" r:id="rId82" display="mailto:invest@voskhod.vc" xr:uid="{702F7933-E9CF-064D-9CC8-6065D575A4E0}"/>
+    <hyperlink ref="D109" r:id="rId83" display="mailto:invest@skcapital.ru" xr:uid="{F4986501-FA20-FB4F-B50C-418D78037BC0}"/>
+    <hyperlink ref="D110" r:id="rId84" display="mailto:invest@trinfico.ru" xr:uid="{5D6D6F2C-B6D6-BA47-B925-58746385FCC0}"/>
+    <hyperlink ref="D111" r:id="rId85" display="mailto:invest@1147group.ru" xr:uid="{384280A8-BE12-5F4A-9A70-0AB64BAC093B}"/>
+    <hyperlink ref="D112" r:id="rId86" display="mailto:invest@alfin.am" xr:uid="{770D3C6B-7F7D-6B49-B087-38479CC152BF}"/>
+    <hyperlink ref="D113" r:id="rId87" display="mailto:invest@cfcm.ru" xr:uid="{10D4B88E-FBCF-2E41-A1A8-30BB6DCEC0E1}"/>
+    <hyperlink ref="D114" r:id="rId88" display="mailto:invest@fordewind.ru" xr:uid="{04D30E16-4C38-284F-87CD-E477B504C7AA}"/>
+    <hyperlink ref="D115" r:id="rId89" display="mailto:invest@aquilainvest.ru" xr:uid="{9DD8A7AA-8099-8649-88B7-06BE0652A014}"/>
+    <hyperlink ref="D116" r:id="rId90" display="mailto:invest@volga-group.ru" xr:uid="{C9BF6FF8-DC26-8F4E-9296-78AE40E58A31}"/>
+    <hyperlink ref="D117" r:id="rId91" display="mailto:invest@alfagroup.ru" xr:uid="{8339C842-6F36-6640-AAFD-5ADBEADCD1BA}"/>
+    <hyperlink ref="D118" r:id="rId92" display="mailto:invest@phystechventures.ru" xr:uid="{D972B136-F670-EA40-80B1-E714C6D07B60}"/>
+    <hyperlink ref="D119" r:id="rId93" display="mailto:invest@ucm.ru" xr:uid="{8DA14F71-EE73-504F-BC1F-8C2CC7EF3DB6}"/>
+    <hyperlink ref="D120" r:id="rId94" display="mailto:invest@polyus.com" xr:uid="{79E9CFEF-81A0-FB4B-84F7-C1F943E1C996}"/>
+    <hyperlink ref="D121" r:id="rId95" display="mailto:partners@frii.ru" xr:uid="{3DF8B87A-9F44-6644-9BF1-BD271FB5ACAB}"/>
+    <hyperlink ref="D122" r:id="rId96" display="mailto:invest@mvf.ru" xr:uid="{87D3E38C-5249-374C-89D8-795085E7C669}"/>
+    <hyperlink ref="D123" r:id="rId97" display="mailto:invest@impactcapital.ru" xr:uid="{D4767112-BB68-7940-A82D-8C9ED793620D}"/>
+    <hyperlink ref="D124" r:id="rId98" display="mailto:info@nti.ru" xr:uid="{D7155472-CBBF-594C-BF64-154BA6E27E0E}"/>
+    <hyperlink ref="D125" r:id="rId99" display="mailto:invest@iskraventures.ru" xr:uid="{D806CC36-AC72-F64E-B2C2-121C3A90C754}"/>
+    <hyperlink ref="D126" r:id="rId100" display="mailto:startups@bee-hive.ru" xr:uid="{1FCCA894-2482-7843-BA8B-0A0987616D0D}"/>
+    <hyperlink ref="D127" r:id="rId101" display="mailto:startups@malina.vc" xr:uid="{66EA8F9B-BA16-B840-9F42-10D792F336A2}"/>
+    <hyperlink ref="D128" r:id="rId102" display="mailto:hello@friends.vc" xr:uid="{61F647B8-0463-B94E-B926-E5554BE19370}"/>
+    <hyperlink ref="D129" r:id="rId103" display="mailto:invest@voskhod.vc" xr:uid="{750D5EED-5F83-6244-B60A-DF11BA4B0986}"/>
+    <hyperlink ref="D130" r:id="rId104" display="mailto:iz@tealtechcapital.com" xr:uid="{41AD0E28-95E7-BF41-B67F-B3272F26FF4D}"/>
+    <hyperlink ref="D131" r:id="rId105" display="mailto:invest@stcapital.ru" xr:uid="{7668B93D-D68C-D749-A7C9-0672D192E67E}"/>
+    <hyperlink ref="D132" r:id="rId106" display="mailto:info@softlinevp.com" xr:uid="{2E53CEBE-845A-1F49-9209-67CA9A691772}"/>
+    <hyperlink ref="D133" r:id="rId107" display="mailto:invest@signal.vc" xr:uid="{0C8DF45C-9488-6048-88E1-3725E037C53D}"/>
+    <hyperlink ref="D134" r:id="rId108" display="mailto:invest@skolkovo.vc" xr:uid="{4BB4212B-F7DB-FD49-A427-B039BBBBE32F}"/>
+    <hyperlink ref="D135" r:id="rId109" display="mailto:invest@lanitventures.ru" xr:uid="{7CE1828F-D516-C24A-B5E9-03EEDBC772E2}"/>
+    <hyperlink ref="D136" r:id="rId110" display="mailto:invest@staminavc.ru" xr:uid="{E0456E3E-28E4-B34D-B7D0-57CADEE14D3A}"/>
+    <hyperlink ref="D137" r:id="rId111" display="mailto:invest@3streams.ru" xr:uid="{BE148DB4-8B61-2B4C-8554-52CF89D0DBA8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C120" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 

</xml_diff>